<commit_message>
Sync multiomics recipes catalog
</commit_message>
<xml_diff>
--- a/RECIPES.xlsx
+++ b/RECIPES.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:J9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -678,6 +678,182 @@
       <c r="J5" s="2" t="inlineStr">
         <is>
           <t>Compose-up RETROFIT candidate: CellBender / remote execution are optional layers. Needs CUDA for CellBender (see AGENTS.md CUDA policy).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>catatac-trimodal-e2e-smoke</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>CAT-ATAC trimodal downsample E2E — RNA + ATAC + guide</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>trimodal</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>scripts/run_catatac_trimodal_downsample_smoke.sh</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr"/>
+      <c r="F6" s="2" t="inlineStr"/>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>multiomics-suite/docs/datasets/e2e_downsample_smoke_runs_20260617.md</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Paper-facing L1 reproducibility smoke. Runs the STAR-suite CAT-ATAC trimodal harness on a 100k downsample and then runs the standalone Signac/MACS BED-profile ATAC peak-MEX pass from the sidecar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>dogma-hiv-four-arm-e2e-smoke</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>DOGMA-HIV four-arm downsample E2E — RNA + ATAC + ADT + HIV state</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>four-ome</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>scripts/run_hiv_dogma_four_arm_downsample_smoke.sh</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr"/>
+      <c r="F7" s="2" t="inlineStr"/>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>multiomics-suite/docs/datasets/e2e_downsample_smoke_runs_20260617.md</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>Paper-facing L1 reproducibility smoke. Materializes matched physical first-N FASTQs for all FASTQ arms, runs the STAR-suite DOGMA table-backed four-arm harness, and then runs the standalone Signac/MACS BED-profile ATAC peak-MEX pass from the sidecar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>trimodal-qc-report</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Trimodal MuData QC report — RNA + ATAC + guide</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>multiomics-report</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>scripts/generate_trimodal_qc.py</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr"/>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>multiomics-suite downstream MuData report recipes</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>Downstream-from-MuData report recipe for the L4 agentic composability surface. It renders the unified trimodal QC from an assembled MuData object.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>four-factor-qc-report</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Four-factor MuData QC report — RNA + ATAC + protein + identity</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>multiomics-report</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>scripts/generate_four_factor_qc.py</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr"/>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>multiomics-suite downstream MuData report recipes</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>Downstream-from-MuData report recipe for the L4 agentic composability surface. It renders protein-aware four-factor QC from an assembled MuData object with optional guide/hash/state identity modalities.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Multiomics MuData builder catalog entry
</commit_message>
<xml_diff>
--- a/RECIPES.xlsx
+++ b/RECIPES.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:J10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -854,6 +854,50 @@
       <c r="J9" s="2" t="inlineStr">
         <is>
           <t>Downstream-from-MuData report recipe for the L4 agentic composability surface. It renders protein-aware four-factor QC from an assembled MuData object with optional guide/hash/state identity modalities.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>multiome-mudata-builder</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Multiome MuData builder — RNA + ATAC plus optional protein/guide/hash/state</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>multiomics-builder</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>scripts/build_multiome_mudata.py</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr"/>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>multiomics-suite/docs/runbooks/RUNBOOK_MULTIOME_MEX_MUDATA_20260516.md</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>Public object-assembly recipe for Multiomics Suite outputs. Builds MuData from RNA and ATAC MEX inputs and can add protein/ADT, CRISPR guide, HTO/hash, and table-backed state modalities with feature-library provenance.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Link recipes to composition evidence
</commit_message>
<xml_diff>
--- a/RECIPES.xlsx
+++ b/RECIPES.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J10"/>
+  <dimension ref="A1:K10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -441,8 +441,9 @@
     <col width="22" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="60" customWidth="1" min="10" max="10"/>
+    <col width="48" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="60" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -488,10 +489,15 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
+          <t>composition examples</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
           <t>status</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
@@ -540,10 +546,15 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
+          <t>composition_morphic_jax_multiome01_20260517t183219z_star_multiome_prod_globus</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
           <t>current</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>Compose-up reference recipe. matrices-peaks = apples-to-apples with Cell Ranger ARC --no-bam + a Signac/MACS peak re-call; full = MorPhiC production superset (adds Velocyto + GEX BAM + Y/noY + remote downstream). Optional --chromap-macs3-frag-qvalue enables libchromap/MACS3 q-value peak selection without changing the default p-value mode.</t>
         </is>
@@ -584,10 +595,15 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
+          <t>composition_morphic_jax_multiome01_20260517t183219z_star_multiome_prod_globus</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
           <t>project-wrapper</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr">
+      <c r="K3" s="2" t="inlineStr">
         <is>
           <t>Thin project wrapper of the multiome engine with the verified jax_multiome01 production parameters. Use the generic engine for new work.</t>
         </is>
@@ -628,10 +644,15 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
+          <t>composition_morphic_jax_scrnaseq02_20260522t135526z_ocm_prod_handoff</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
           <t>current</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr">
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>Compose-up RETROFIT candidate: Velocyto / BAM / remote downstream are optional layers that should become --profile/flags.</t>
         </is>
@@ -670,12 +691,13 @@
           <t>runs/msk_30ko_revised</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="I5" s="2" t="inlineStr"/>
+      <c r="J5" s="2" t="inlineStr">
         <is>
           <t>current</t>
         </is>
       </c>
-      <c r="J5" s="2" t="inlineStr">
+      <c r="K5" s="2" t="inlineStr">
         <is>
           <t>Compose-up RETROFIT candidate: CellBender / remote execution are optional layers. Needs CUDA for CellBender (see AGENTS.md CUDA policy).</t>
         </is>
@@ -714,12 +736,13 @@
           <t>multiomics-suite/docs/datasets/e2e_downsample_smoke_runs_20260617.md</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="I6" s="2" t="inlineStr"/>
+      <c r="J6" s="2" t="inlineStr">
         <is>
           <t>current</t>
         </is>
       </c>
-      <c r="J6" s="2" t="inlineStr">
+      <c r="K6" s="2" t="inlineStr">
         <is>
           <t>Paper-facing L1 reproducibility smoke. Runs the STAR-suite CAT-ATAC trimodal harness on a 100k downsample and then runs the standalone Signac/MACS BED-profile ATAC peak-MEX pass from the sidecar.</t>
         </is>
@@ -758,12 +781,13 @@
           <t>multiomics-suite/docs/datasets/e2e_downsample_smoke_runs_20260617.md</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr"/>
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>current</t>
         </is>
       </c>
-      <c r="J7" s="2" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>Paper-facing L1 reproducibility smoke. Materializes matched physical first-N FASTQs for all FASTQ arms, runs the STAR-suite DOGMA table-backed four-arm harness, and then runs the standalone Signac/MACS BED-profile ATAC peak-MEX pass from the sidecar.</t>
         </is>
@@ -802,12 +826,13 @@
           <t>multiomics-suite downstream MuData report recipes</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="I8" s="2" t="inlineStr"/>
+      <c r="J8" s="2" t="inlineStr">
         <is>
           <t>current</t>
         </is>
       </c>
-      <c r="J8" s="2" t="inlineStr">
+      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>Downstream-from-MuData report recipe for the L4 agentic composability surface. It renders the unified trimodal QC from an assembled MuData object.</t>
         </is>
@@ -846,12 +871,13 @@
           <t>multiomics-suite downstream MuData report recipes</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="I9" s="2" t="inlineStr"/>
+      <c r="J9" s="2" t="inlineStr">
         <is>
           <t>current</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr">
+      <c r="K9" s="2" t="inlineStr">
         <is>
           <t>Downstream-from-MuData report recipe for the L4 agentic composability surface. It renders protein-aware four-factor QC from an assembled MuData object with optional guide/hash/state identity modalities.</t>
         </is>
@@ -890,12 +916,13 @@
           <t>multiomics-suite/docs/runbooks/RUNBOOK_MULTIOME_MEX_MUDATA_20260516.md</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="I10" s="2" t="inlineStr"/>
+      <c r="J10" s="2" t="inlineStr">
         <is>
           <t>current</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr">
+      <c r="K10" s="2" t="inlineStr">
         <is>
           <t>Public object-assembly recipe for Multiomics Suite outputs. Builds MuData from RNA and ATAC MEX inputs and can add protein/ADT, CRISPR guide, HTO/hash, and table-backed state modalities with feature-library provenance.</t>
         </is>

</xml_diff>